<commit_message>
Publish batch 14 and queue cleanup updates
</commit_message>
<xml_diff>
--- a/assets/downloads/world500_current_status_distribution_zh.xlsx
+++ b/assets/downloads/world500_current_status_distribution_zh.xlsx
@@ -443,12 +443,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="38" customWidth="1" min="6" max="6"/>
@@ -551,11 +551,11 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>65.0%</t>
+          <t>66.4%</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>已发布批次：batch_01, batch_02, batch_03, batch_04, batch_05, batch_06, batch_07, batch_08, batch_09, batch_10, batch_11, batch_12, batch_13</t>
+          <t>已发布批次：batch_01, batch_02, batch_03, batch_04, batch_05, batch_06, batch_07, batch_08, batch_09, batch_10, batch_11, batch_12, batch_13, batch_14</t>
         </is>
       </c>
     </row>
@@ -580,35 +580,35 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>待发布</t>
+          <t>未匹配待补库/复核</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>已匹配且完成抽取/证据，但尚未进入已发布批次</t>
+          <t>库内无母公司主报告</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>7</v>
+        <v>161</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>1.4%</t>
+          <t>32.2%</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>已完成报告匹配并进入批次编排，但尚未纳入已发布批次成果。</t>
+          <t>当前库存中未发现可安全归属母公司的正式主报告文件。</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>优先完成待发布批次的正式出图、指标汇总和站点接入。</t>
+          <t>保持未匹配状态，按高价值对象继续二次检索补库。</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>待发布批次：batch_14</t>
+          <t>来源：world500_unmatched_diagnosis.csv 开放未决匹配诊断</t>
         </is>
       </c>
     </row>
@@ -623,25 +623,25 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>库内无母公司主报告</t>
+          <t>仅发现子公司/关联主体文件</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>161</v>
+        <v>6</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>32.2%</t>
+          <t>1.2%</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>当前库存中未发现可安全归属母公司的正式主报告文件。</t>
+          <t>仅发现上市子公司或关联经营主体材料，不能替代母公司主报告。</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>保持未匹配状态，按高价值对象继续二次检索补库。</t>
+          <t>人工复核是否补采母公司主报告；现有关联主体文件不直接入主图谱。</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -661,94 +661,56 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>仅发现子公司/关联主体文件</t>
+          <t>人工判定驳回的错误匹配</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>1.2%</t>
+          <t>0.2%</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>仅发现上市子公司或关联经营主体材料，不能替代母公司主报告。</t>
+          <t>已存在人工驳回记录，确认当前候选文件不能安全匹配到母公司主报告。</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>人工复核是否补采母公司主报告；现有关联主体文件不直接入主图谱。</t>
+          <t>保留 rejection note，不做硬匹配。</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>来源：world500_unmatched_diagnosis.csv 开放未决匹配诊断</t>
+          <t>来源：world500_report_catalog.csv 中 match_status=unmatched_manual</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>5</v>
-      </c>
+      <c r="A9" s="2" t="inlineStr"/>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>未匹配待补库/复核</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>人工判定驳回的错误匹配</t>
-        </is>
-      </c>
+          <t>合计</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr"/>
       <c r="D9" s="2" t="n">
-        <v>1</v>
+        <v>500</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>0.2%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>已存在人工驳回记录，确认当前候选文件不能安全匹配到母公司主报告。</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>保留 rejection note，不做硬匹配。</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>来源：world500_report_catalog.csv 中 match_status=unmatched_manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>合计</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="n">
-        <v>500</v>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
           <t>500 家世界500强正式推进对象。</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update world500 queue, axis backfill, and retrieval batch 02 assets
</commit_message>
<xml_diff>
--- a/assets/downloads/world500_current_status_distribution_zh.xlsx
+++ b/assets/downloads/world500_current_status_distribution_zh.xlsx
@@ -1123,80 +1123,80 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>页级抽取质量待复核</t>
+          <t>报告匹配未解决</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>extract_quality</t>
+          <t>report_unmatched</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>288</v>
+        <v>167</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>45.1%</t>
+          <t>53.7%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>报告匹配未解决</t>
+          <t>关键证据缺口待补齐</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>report_unmatched</t>
+          <t>evidence_gap</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>167</v>
+        <v>87</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>26.1%</t>
+          <t>28.0%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>关键证据缺口待补齐</t>
+          <t>匹配结果抽检</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>evidence_gap</t>
+          <t>match_spotcheck</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>133</v>
+        <v>51</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>20.8%</t>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>匹配结果抽检</t>
+          <t>页级抽取质量待复核</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>match_spotcheck</t>
+          <t>extract_quality</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>51</v>
+        <v>6</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>8.0%</t>
+          <t>1.9%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Integrate BBVA and Lloyds into world500 pipeline
</commit_message>
<xml_diff>
--- a/assets/downloads/world500_current_status_distribution_zh.xlsx
+++ b/assets/downloads/world500_current_status_distribution_zh.xlsx
@@ -551,11 +551,11 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>332</v>
+        <v>351</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>66.4%</t>
+          <t>70.2%</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>已发布批次：batch_01, batch_02, batch_03, batch_04, batch_05, batch_06, batch_07, batch_08, batch_09, batch_10, batch_11, batch_12, batch_13, batch_14</t>
+          <t>已发布批次：batch_01, batch_02, batch_03, batch_04, batch_05, batch_06, batch_07, batch_08, batch_09, batch_10, batch_11, batch_12, batch_13, batch_14, batch_15</t>
         </is>
       </c>
     </row>
@@ -589,11 +589,11 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>161</v>
+        <v>141</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>32.2%</t>
+          <t>28.2%</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -665,11 +665,11 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>0.2%</t>
+          <t>0.4%</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -810,16 +810,16 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>161</v>
+        <v>141</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>32.2%</t>
+          <t>28.2%</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>96.4%</t>
+          <t>95.9%</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -849,7 +849,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>3.6%</t>
+          <t>4.1%</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -930,11 +930,11 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>0.2%</t>
+          <t>0.4%</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
@@ -1063,11 +1063,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
@@ -1132,11 +1132,11 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>167</v>
+        <v>146</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>53.7%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
@@ -1152,11 +1152,11 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>28.0%</t>
+          <t>31.5%</t>
         </is>
       </c>
     </row>
@@ -1176,27 +1176,47 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>17.5%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>页级抽取质量待复核</t>
+          <t>page_extract_missing</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>extract_quality</t>
+          <t>page_extract_missing</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>1.9%</t>
+          <t>0.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>report_match_review</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>report_match_review</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>0.3%</t>
         </is>
       </c>
     </row>

</xml_diff>